<commit_message>
PVC · revisión de coherencia: dossier armonizado, D4 ES/EN = exportación del tablero (V5.29)
Un solo código de edición (PVC-F4-2026) y una sola etiqueta de versión (v2.1.1);
D2/D3/D0/D1 describen la publicación con huella en BCP · PVC y los ciclos
semanales; el D4 lleva los tres KPIs y la escalera FCA/CIP/DDP con el mismo
esqueleto que «Exportar Reporte» en español e inglés; redondeo comercial en el
motor Python; guardián qa-pvc-tablero; tablas con el estilo del panel; un solo
camino de publicación.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/pvc/v2.1.1/PVC_Calculadora_CTCx.xlsx
+++ b/docs/pvc/v2.1.1/PVC_Calculadora_CTCx.xlsx
@@ -592,7 +592,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Método: PVC-D2 v2.1 · Datos: PVC-D1 v2.1 · Edición precargada: PVC-F4 2026 (corte 4-sep-2026, reedición v2.1 9-sep-2026 con series oficiales). Comparador: precio efectivo de cooperativa (PEC) + prima objetivo.</t>
+          <t>Método: PVC-D2 v2.1.1 · Datos: PVC-D1 v2.1.1 · Edición precargada: PVC-F4-2026 (corte 4-sep-2026, reedición v2.1 9-sep-2026 con series oficiales). Comparador: precio efectivo de cooperativa (PEC) + prima objetivo.</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>PVC-F4-2026-v2.1</t>
+          <t>PVC-F4-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>D2 §8 (decisión CTCx v2.0)</t>
+          <t>D2 §8 (decisión CTCx v2.0.1)</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cálculo del PVC v2.0 (D2 §4–7)</t>
+          <t>Cálculo del PVC (D2 §4–7)</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Escalera de calidad CTCx v2.0 (D2 §8) · columnas FCA/CIP desde la hoja Pila_de_precios (D2 §13.1)</t>
+          <t>Escalera de calidad CTCx (D2 §8) · columnas FCA/CIP desde la hoja Pila_de_precios (D2 §13.1)</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Calendario v2.0 · franjas de venta 2027 (D2 §7.2)</t>
+          <t>Calendario · franjas de venta 2027 (D2 §7.2)</t>
         </is>
       </c>
     </row>

</xml_diff>